<commit_message>
Revision of right label definitions
</commit_message>
<xml_diff>
--- a/projects/project-3/assignment/src/data/ccot-time-structural-matches.xlsx
+++ b/projects/project-3/assignment/src/data/ccot-time-structural-matches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cappa\Ontology-Tradecraft\projects\project-3\assignment\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19FD6D46-8E7B-4DAA-AF47-E0BF0ECC8E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FE20CF-4EA4-4015-9055-7805F391C01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -654,7 +654,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H101"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -694,7 +693,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -720,7 +719,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -746,7 +745,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -772,7 +771,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -798,7 +797,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -824,7 +823,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -850,7 +849,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>73</v>
       </c>
@@ -876,7 +875,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -902,7 +901,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -928,7 +927,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -954,7 +953,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -980,7 +979,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1006,7 +1005,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1032,7 +1031,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -1110,7 +1109,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -1136,7 +1135,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>55</v>
       </c>
@@ -1162,7 +1161,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>52</v>
       </c>
@@ -1188,7 +1187,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -1214,7 +1213,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>52</v>
       </c>
@@ -1240,7 +1239,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -1266,7 +1265,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -1292,7 +1291,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -1318,7 +1317,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>61</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>61</v>
       </c>
@@ -1370,7 +1369,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>61</v>
       </c>
@@ -1396,7 +1395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -1422,7 +1421,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>61</v>
       </c>
@@ -1474,7 +1473,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>67</v>
       </c>
@@ -1500,7 +1499,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>67</v>
       </c>
@@ -1526,7 +1525,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -1552,7 +1551,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>67</v>
       </c>
@@ -1578,7 +1577,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>67</v>
       </c>
@@ -1604,7 +1603,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>67</v>
       </c>
@@ -1630,7 +1629,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>49</v>
       </c>
@@ -1656,7 +1655,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>49</v>
       </c>
@@ -1682,7 +1681,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -1708,7 +1707,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>49</v>
       </c>
@@ -1734,7 +1733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>49</v>
       </c>
@@ -1760,7 +1759,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="43" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>49</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>64</v>
       </c>
@@ -1812,7 +1811,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
         <v>64</v>
       </c>
@@ -1838,7 +1837,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>64</v>
       </c>
@@ -1864,7 +1863,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>64</v>
       </c>
@@ -1890,7 +1889,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>64</v>
       </c>
@@ -1916,7 +1915,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
         <v>64</v>
       </c>
@@ -1942,7 +1941,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>76</v>
       </c>
@@ -1968,7 +1967,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>76</v>
       </c>
@@ -1994,7 +1993,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>76</v>
       </c>
@@ -2020,7 +2019,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>76</v>
       </c>
@@ -2046,7 +2045,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>76</v>
       </c>
@@ -2072,7 +2071,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>76</v>
       </c>
@@ -2098,7 +2097,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>70</v>
       </c>
@@ -2124,7 +2123,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
         <v>70</v>
       </c>
@@ -2150,7 +2149,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>70</v>
       </c>
@@ -2176,7 +2175,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>70</v>
       </c>
@@ -2202,7 +2201,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>70</v>
       </c>
@@ -2228,7 +2227,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>70</v>
       </c>
@@ -2254,7 +2253,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>34</v>
       </c>
@@ -2280,7 +2279,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>34</v>
       </c>
@@ -2306,7 +2305,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>34</v>
       </c>
@@ -2332,7 +2331,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>34</v>
       </c>
@@ -2358,7 +2357,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
         <v>34</v>
       </c>
@@ -2384,7 +2383,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>34</v>
       </c>
@@ -2410,7 +2409,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="68" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>43</v>
       </c>
@@ -2436,7 +2435,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
         <v>43</v>
       </c>
@@ -2462,7 +2461,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>43</v>
       </c>
@@ -2488,7 +2487,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>43</v>
       </c>
@@ -2514,7 +2513,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>43</v>
       </c>
@@ -2540,7 +2539,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="73" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
         <v>43</v>
       </c>
@@ -2566,7 +2565,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>46</v>
       </c>
@@ -2592,7 +2591,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>46</v>
       </c>
@@ -2618,7 +2617,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>46</v>
       </c>
@@ -2644,7 +2643,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>46</v>
       </c>
@@ -2670,7 +2669,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>46</v>
       </c>
@@ -2696,7 +2695,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>46</v>
       </c>
@@ -2722,7 +2721,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>40</v>
       </c>
@@ -2748,7 +2747,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>40</v>
       </c>
@@ -2826,7 +2825,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>40</v>
       </c>
@@ -2852,7 +2851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>40</v>
       </c>
@@ -2878,7 +2877,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="86" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>58</v>
       </c>
@@ -2904,7 +2903,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>58</v>
       </c>
@@ -2930,7 +2929,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>58</v>
       </c>
@@ -2956,7 +2955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>58</v>
       </c>
@@ -2982,7 +2981,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>58</v>
       </c>
@@ -3008,7 +3007,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>58</v>
       </c>
@@ -3034,7 +3033,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" spans="1:8" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>8</v>
       </c>
@@ -3086,7 +3085,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -3112,7 +3111,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -3138,7 +3137,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>8</v>
       </c>
@@ -3164,7 +3163,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>8</v>
       </c>
@@ -3206,11 +3205,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B97" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <colorFilter dxfId="0"/>
-    </filterColumn>
-  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H97">
     <sortCondition ref="B2:B97"/>
   </sortState>

</xml_diff>